<commit_message>
Added more to data folder and some cartoonish rule curve plots for the workshop
</commit_message>
<xml_diff>
--- a/data/common_data/Reservoirs.xlsx
+++ b/data/common_data/Reservoirs.xlsx
@@ -1,25 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Willamette_Flow_Frequency_2021\common_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Python\Willamette_FIRO\data\common_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43242E38-A385-464B-8F5F-47D01D527E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A21550-59BE-4A66-83F8-E494AB2CA51F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{FC561D18-D4CD-4EFF-9AED-16460E500202}"/>
+    <workbookView xWindow="-108" yWindow="-84" windowWidth="23256" windowHeight="13872" xr2:uid="{FC561D18-D4CD-4EFF-9AED-16460E500202}"/>
   </bookViews>
   <sheets>
     <sheet name="Reservoirs" sheetId="2" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Reservoirs!$A$6:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Reservoirs!$A$6:$P$17</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,9 +40,10 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Ryan Cahill</author>
+    <author>Cahill, Ryan J CIV USARMY CENWP (USA)</author>
   </authors>
   <commentList>
-    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{22014E07-8B99-44EC-A90F-5E9619EE5AEA}">
+    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{22014E07-8B99-44EC-A90F-5E9619EE5AEA}">
       <text>
         <r>
           <rPr>
@@ -53,7 +51,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Ryan Cahill:</t>
         </r>
@@ -62,14 +60,14 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Intended to be the lowest operational outlet, not the minimum conservation. "RO Invert Elevation" from WillametteReservoirStatistics.xlsx unless otherwise notes</t>
         </r>
       </text>
     </comment>
-    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{7703FE8C-6CF1-4FE3-8C3F-AF5F8DBE2D98}">
+    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{7703FE8C-6CF1-4FE3-8C3F-AF5F8DBE2D98}">
       <text>
         <r>
           <rPr>
@@ -77,7 +75,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Ryan Cahill:</t>
         </r>
@@ -86,14 +84,14 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 "Full Pool" from WillametteReservoirStatistics.xlsx</t>
         </r>
       </text>
     </comment>
-    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{B8BE2FDC-7F18-445D-A446-015930C441B8}">
+    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{B8BE2FDC-7F18-445D-A446-015930C441B8}">
       <text>
         <r>
           <rPr>
@@ -101,7 +99,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Ryan Cahill:</t>
         </r>
@@ -110,14 +108,14 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 "Min Conservation Pool" from WillametteReservoirStatistics.xlsx</t>
         </r>
       </text>
     </comment>
-    <comment ref="G6" authorId="0" shapeId="0" xr:uid="{F742BCCB-83A4-450B-9078-11FABA03805F}">
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{F742BCCB-83A4-450B-9078-11FABA03805F}">
       <text>
         <r>
           <rPr>
@@ -125,7 +123,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Ryan Cahill:</t>
         </r>
@@ -134,14 +132,14 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 "Max Conservation Pool" from WillametteReservoirStatistics.xlsx</t>
         </r>
       </text>
     </comment>
-    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{43748031-8996-4C09-89BF-3329905CB58D}">
+    <comment ref="H6" authorId="1" shapeId="0" xr:uid="{702BC60D-34EE-4B71-A460-F1801BDF0A23}">
       <text>
         <r>
           <rPr>
@@ -149,8 +147,104 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Cahill, Ryan J CIV USARMY CENWP (USA):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Deep drawdown target as of 8/27/2026</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J6" authorId="1" shapeId="0" xr:uid="{D5D4704A-B2A8-4B4D-BBFD-698BBD4724E8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Cahill, Ryan J CIV USARMY CENWP (USA):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Dam Safety IRRM for seismic pool restriction</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O6" authorId="1" shapeId="0" xr:uid="{CCFF0DCB-1040-4B9E-863B-7B9E2D9C3DC2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
+          <t>Cahill, Ryan J CIV USARMY CENWP (USA):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Sourced from "High flow period" min flow in WillametteReservoirStatistics.xlsx. This is not BiOp min.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I9" authorId="1" shapeId="0" xr:uid="{8175DB5E-5454-4436-8701-8A460BD0C610}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Cahill, Ryan J CIV USARMY CENWP (USA):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+From WCM, listed as "Minimum Pool". Inactive storage of 9,500 ac-ft listed matches up with Water_Control_Diagrams.xlsx, but it shows it down to 670 ft</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{43748031-8996-4C09-89BF-3329905CB58D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t>Ryan Cahill:</t>
         </r>
         <r>
@@ -158,14 +252,14 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Diversion Tunnel Invert</t>
         </r>
       </text>
     </comment>
-    <comment ref="D16" authorId="0" shapeId="0" xr:uid="{B74998C1-0D4D-4384-A8B6-4049C2E287F7}">
+    <comment ref="I12" authorId="1" shapeId="0" xr:uid="{3D688B94-6BD8-4251-B325-6FF1D9E901E2}">
       <text>
         <r>
           <rPr>
@@ -173,7 +267,55 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
+          </rPr>
+          <t>Cahill, Ryan J CIV USARMY CENWP (USA):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Delayed Refill drawdown target</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I14" authorId="1" shapeId="0" xr:uid="{154B68AA-68E9-465F-B684-56D047755F4C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Cahill, Ryan J CIV USARMY CENWP (USA):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+"Low Point in Reservoir" per WCM. Says 2,800 of storage, which matches up with Water_Control_Manuals.xlsx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C16" authorId="0" shapeId="0" xr:uid="{B74998C1-0D4D-4384-A8B6-4049C2E287F7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>Ryan Cahill:</t>
         </r>
@@ -182,14 +324,14 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 No ROs, Turbine Invert elevation. Also spillway crest.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D17" authorId="0" shapeId="0" xr:uid="{80A9B8BD-2B5B-47B7-A289-D2D0EBE3072A}">
+    <comment ref="I16" authorId="0" shapeId="0" xr:uid="{63C6247A-B61C-4FF2-A4D4-EC6FD83FA72D}">
       <text>
         <r>
           <rPr>
@@ -197,7 +339,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Ryan Cahill:</t>
         </r>
@@ -206,7 +348,31 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+No ROs, Turbine Invert elevation. Also spillway crest.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C17" authorId="0" shapeId="0" xr:uid="{80A9B8BD-2B5B-47B7-A289-D2D0EBE3072A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Ryan Cahill:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Upper RO Invert</t>
@@ -218,7 +384,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>The top 5 lines of this sheet are reserved for descriptive comments. The headers should be in line 6 and data in row 7.</t>
   </si>
@@ -268,51 +434,12 @@
     <t>ReservoirName</t>
   </si>
   <si>
-    <t>CBT_Code</t>
-  </si>
-  <si>
     <t>MinElev</t>
   </si>
   <si>
-    <t>MaxElev</t>
-  </si>
-  <si>
     <t>MinConElev</t>
   </si>
   <si>
-    <t>HCR</t>
-  </si>
-  <si>
-    <t>LOP</t>
-  </si>
-  <si>
-    <t>FAL</t>
-  </si>
-  <si>
-    <t>DOR</t>
-  </si>
-  <si>
-    <t>COT</t>
-  </si>
-  <si>
-    <t>CGR</t>
-  </si>
-  <si>
-    <t>BLU</t>
-  </si>
-  <si>
-    <t>FRN</t>
-  </si>
-  <si>
-    <t>GPR</t>
-  </si>
-  <si>
-    <t>FOS</t>
-  </si>
-  <si>
-    <t>DET</t>
-  </si>
-  <si>
     <t>This is typically read by the scripts dealing with Synthetic inputs to ResSim and the starting pool storage.</t>
   </si>
   <si>
@@ -320,13 +447,43 @@
   </si>
   <si>
     <t>MaxConElev</t>
+  </si>
+  <si>
+    <t>IRRMElev</t>
+  </si>
+  <si>
+    <t>NormalEvacRate</t>
+  </si>
+  <si>
+    <t>MaxEvacRate</t>
+  </si>
+  <si>
+    <t>SpillwayCrest</t>
+  </si>
+  <si>
+    <t>MinPowerPool</t>
+  </si>
+  <si>
+    <t>Data sourced from WillametteReservoirStatistics.xlsx unless otherwise noted</t>
+  </si>
+  <si>
+    <t>FullPoolElev</t>
+  </si>
+  <si>
+    <t>InactivePool</t>
+  </si>
+  <si>
+    <t>DrawdownPool</t>
+  </si>
+  <si>
+    <t>MinFlowFlood</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -346,9 +503,22 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <charset val="1"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
@@ -395,156 +565,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="stats"/>
-      <sheetName val="flows"/>
-      <sheetName val="Boat Ramps"/>
-      <sheetName val="fill&amp;draft"/>
-      <sheetName val="ramp rates"/>
-      <sheetName val="MinFlow"/>
-      <sheetName val="Schematic"/>
-      <sheetName val="pool elevations"/>
-      <sheetName val="Pool of Record"/>
-      <sheetName val="May15 Stg"/>
-      <sheetName val="RuleCurve"/>
-      <sheetName val="FOS Fish Weir"/>
-      <sheetName val="temps"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="4">
-          <cell r="C4" t="str">
-            <v>HCR</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v>LOP</v>
-          </cell>
-          <cell r="E4" t="str">
-            <v>DEX</v>
-          </cell>
-          <cell r="F4" t="str">
-            <v>FAL</v>
-          </cell>
-          <cell r="G4" t="str">
-            <v>COT</v>
-          </cell>
-          <cell r="H4" t="str">
-            <v>DOR</v>
-          </cell>
-          <cell r="I4" t="str">
-            <v>FRN</v>
-          </cell>
-          <cell r="J4" t="str">
-            <v>CGR</v>
-          </cell>
-          <cell r="K4" t="str">
-            <v>BLU</v>
-          </cell>
-          <cell r="L4" t="str">
-            <v>GPR</v>
-          </cell>
-          <cell r="M4" t="str">
-            <v>FOS</v>
-          </cell>
-          <cell r="N4" t="str">
-            <v>DET</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="C10">
-            <v>1543</v>
-          </cell>
-          <cell r="D10">
-            <v>929</v>
-          </cell>
-          <cell r="E10">
-            <v>695</v>
-          </cell>
-          <cell r="F10">
-            <v>834</v>
-          </cell>
-          <cell r="G10">
-            <v>791</v>
-          </cell>
-          <cell r="H10">
-            <v>835</v>
-          </cell>
-          <cell r="I10">
-            <v>375.1</v>
-          </cell>
-          <cell r="J10">
-            <v>1699</v>
-          </cell>
-          <cell r="K10">
-            <v>1357</v>
-          </cell>
-          <cell r="L10">
-            <v>1015</v>
-          </cell>
-          <cell r="M10">
-            <v>641</v>
-          </cell>
-          <cell r="N10">
-            <v>1569</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="C46">
-            <v>1408.75</v>
-          </cell>
-          <cell r="D46">
-            <v>724</v>
-          </cell>
-          <cell r="F46">
-            <v>670</v>
-          </cell>
-          <cell r="G46">
-            <v>719</v>
-          </cell>
-          <cell r="H46">
-            <v>739</v>
-          </cell>
-          <cell r="I46">
-            <v>340</v>
-          </cell>
-          <cell r="J46">
-            <v>1478.75</v>
-          </cell>
-          <cell r="K46">
-            <v>1132</v>
-          </cell>
-          <cell r="L46">
-            <v>745</v>
-          </cell>
-          <cell r="N46" t="str">
-            <v>2@1,335&amp;1260</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -582,7 +606,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -688,7 +712,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -830,7 +854,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -838,37 +862,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DBC2FD2-6A64-426A-9430-3B333C72098D}">
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="7" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" customWidth="1"/>
+    <col min="5" max="11" width="14.44140625" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="14.88671875" customWidth="1"/>
+    <col min="14" max="15" width="16.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -879,295 +910,516 @@
         <v>16</v>
       </c>
       <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" t="s">
-        <v>18</v>
-      </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="H6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" t="s">
+        <v>30</v>
+      </c>
+      <c r="P6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>20</v>
+      <c r="C7" s="1">
+        <v>1408.75</v>
       </c>
       <c r="D7" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C7, [1]stats!$C$4:$N$4,0))</f>
-        <v>1408.75</v>
+        <v>1543</v>
       </c>
       <c r="E7" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C7, [1]stats!$C$4:$N$4,0))</f>
-        <v>1543</v>
+        <v>1448</v>
       </c>
       <c r="F7" s="1">
-        <v>1448</v>
+        <v>1541</v>
       </c>
       <c r="G7" s="1">
-        <v>1541</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1414</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1">
+        <v>1511</v>
+      </c>
+      <c r="K7" s="1">
+        <v>1495.5</v>
+      </c>
+      <c r="L7" s="1">
+        <v>6000</v>
+      </c>
+      <c r="M7" s="1">
+        <v>8000</v>
+      </c>
+      <c r="N7" s="1">
+        <v>1495.5</v>
+      </c>
+      <c r="O7" s="1">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
+      <c r="C8" s="1">
+        <v>724</v>
       </c>
       <c r="D8" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C8, [1]stats!$C$4:$N$4,0))</f>
-        <v>724</v>
+        <v>929</v>
       </c>
       <c r="E8" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C8, [1]stats!$C$4:$N$4,0))</f>
-        <v>929</v>
+        <v>825</v>
       </c>
       <c r="F8" s="1">
-        <v>825</v>
+        <v>926</v>
       </c>
       <c r="G8" s="1">
-        <v>926</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>819</v>
+      </c>
+      <c r="H8" s="1">
+        <v>750</v>
+      </c>
+      <c r="J8" s="1">
+        <v>921</v>
+      </c>
+      <c r="K8" s="1">
+        <v>887.5</v>
+      </c>
+      <c r="L8" s="1">
+        <v>12000</v>
+      </c>
+      <c r="M8" s="1">
+        <v>15000</v>
+      </c>
+      <c r="N8" s="1">
+        <v>887.5</v>
+      </c>
+      <c r="O8" s="1">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>3</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" t="s">
-        <v>22</v>
+      <c r="C9" s="1">
+        <v>670</v>
       </c>
       <c r="D9" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C9, [1]stats!$C$4:$N$4,0))</f>
-        <v>670</v>
+        <v>834</v>
       </c>
       <c r="E9" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C9, [1]stats!$C$4:$N$4,0))</f>
-        <v>834</v>
+        <v>728</v>
       </c>
       <c r="F9" s="1">
-        <v>728</v>
-      </c>
-      <c r="G9" s="1">
         <v>830</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G9" s="1"/>
+      <c r="H9" s="1">
+        <v>680</v>
+      </c>
+      <c r="I9" s="1">
+        <v>673</v>
+      </c>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1">
+        <v>791.6</v>
+      </c>
+      <c r="L9" s="1">
+        <v>3800</v>
+      </c>
+      <c r="M9" s="1">
+        <v>4500</v>
+      </c>
+      <c r="N9" s="1">
+        <v>791.6</v>
+      </c>
+      <c r="O9" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>4</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
       </c>
-      <c r="C10" t="s">
-        <v>23</v>
+      <c r="C10" s="1">
+        <v>739</v>
       </c>
       <c r="D10" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C10, [1]stats!$C$4:$N$4,0))</f>
+        <v>835</v>
+      </c>
+      <c r="E10" s="1">
+        <v>770.5</v>
+      </c>
+      <c r="F10" s="1">
+        <v>832</v>
+      </c>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1">
+        <f>C10</f>
         <v>739</v>
       </c>
-      <c r="E10" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C10, [1]stats!$C$4:$N$4,0))</f>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1">
         <v>835</v>
       </c>
-      <c r="F10" s="1">
-        <v>770.5</v>
-      </c>
-      <c r="G10" s="1">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L10" s="1">
+        <v>2500</v>
+      </c>
+      <c r="M10" s="1">
+        <v>3000</v>
+      </c>
+      <c r="N10" s="1">
+        <v>791</v>
+      </c>
+      <c r="O10" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>5</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
       </c>
-      <c r="C11" t="s">
-        <v>24</v>
+      <c r="C11" s="1">
+        <v>719</v>
       </c>
       <c r="D11" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C11, [1]stats!$C$4:$N$4,0))</f>
+        <v>791</v>
+      </c>
+      <c r="E11" s="1">
+        <v>750</v>
+      </c>
+      <c r="F11" s="1">
+        <v>790</v>
+      </c>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1">
+        <f>C11</f>
         <v>719</v>
       </c>
-      <c r="E11" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C11, [1]stats!$C$4:$N$4,0))</f>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1">
         <v>791</v>
       </c>
-      <c r="F11" s="1">
-        <v>750</v>
-      </c>
-      <c r="G11" s="1">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L11" s="1">
+        <v>4000</v>
+      </c>
+      <c r="M11" s="1">
+        <v>5000</v>
+      </c>
+      <c r="N11" s="1">
+        <v>835</v>
+      </c>
+      <c r="O11" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>6</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
       </c>
-      <c r="C12" t="s">
-        <v>25</v>
+      <c r="C12" s="1">
+        <v>1290</v>
       </c>
       <c r="D12" s="1">
-        <v>1290</v>
+        <v>1699</v>
       </c>
       <c r="E12" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C12, [1]stats!$C$4:$N$4,0))</f>
-        <v>1699</v>
+        <v>1532</v>
       </c>
       <c r="F12" s="1">
-        <v>1532</v>
+        <v>1690</v>
       </c>
       <c r="G12" s="1">
-        <v>1690</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1516</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1">
+        <v>1505</v>
+      </c>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1">
+        <v>1656.75</v>
+      </c>
+      <c r="L12" s="1">
+        <v>3000</v>
+      </c>
+      <c r="M12" s="1">
+        <v>4000</v>
+      </c>
+      <c r="N12" s="1">
+        <v>358.5</v>
+      </c>
+      <c r="O12" s="1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>7</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
       </c>
-      <c r="C13" t="s">
-        <v>26</v>
+      <c r="C13" s="1">
+        <v>1132</v>
       </c>
       <c r="D13" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C13, [1]stats!$C$4:$N$4,0))</f>
-        <v>1132</v>
+        <v>1357</v>
       </c>
       <c r="E13" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C13, [1]stats!$C$4:$N$4,0))</f>
-        <v>1357</v>
+        <v>1180</v>
       </c>
       <c r="F13" s="1">
-        <v>1180</v>
-      </c>
-      <c r="G13" s="1">
         <v>1350</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1">
+        <v>1321</v>
+      </c>
+      <c r="L13" s="1">
+        <v>5000</v>
+      </c>
+      <c r="M13" s="1">
+        <v>6500</v>
+      </c>
+      <c r="N13" s="1">
+        <v>1656.75</v>
+      </c>
+      <c r="O13" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>8</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
       </c>
-      <c r="C14" t="s">
-        <v>27</v>
+      <c r="C14" s="1">
+        <v>340</v>
       </c>
       <c r="D14" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C14, [1]stats!$C$4:$N$4,0))</f>
-        <v>340</v>
+        <v>375.1</v>
       </c>
       <c r="E14" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C14, [1]stats!$C$4:$N$4,0))</f>
-        <v>375.1</v>
+        <v>353</v>
       </c>
       <c r="F14" s="1">
-        <v>353</v>
-      </c>
-      <c r="G14" s="1">
         <v>373.5</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1">
+        <v>347</v>
+      </c>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1">
+        <v>358.5</v>
+      </c>
+      <c r="L14" s="1">
+        <v>3000</v>
+      </c>
+      <c r="M14" s="1">
+        <v>3700</v>
+      </c>
+      <c r="N14" s="1">
+        <v>1321</v>
+      </c>
+      <c r="O14" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>9</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
-      <c r="C15" t="s">
-        <v>28</v>
+      <c r="C15" s="1">
+        <v>745</v>
       </c>
       <c r="D15" s="1">
-        <f>INDEX([1]stats!$C$46:$N$46,MATCH($C15, [1]stats!$C$4:$N$4,0))</f>
-        <v>745</v>
+        <v>1015</v>
       </c>
       <c r="E15" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C15, [1]stats!$C$4:$N$4,0))</f>
-        <v>1015</v>
+        <v>922</v>
       </c>
       <c r="F15" s="1">
-        <v>922</v>
+        <v>1010</v>
       </c>
       <c r="G15" s="1">
-        <v>1010</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>887</v>
+      </c>
+      <c r="H15" s="1">
+        <v>780</v>
+      </c>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1">
+        <v>968.7</v>
+      </c>
+      <c r="L15" s="1">
+        <v>10000</v>
+      </c>
+      <c r="M15" s="1">
+        <v>13000</v>
+      </c>
+      <c r="N15" s="1">
+        <v>968.7</v>
+      </c>
+      <c r="O15" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>10</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
       </c>
-      <c r="C16" t="s">
-        <v>29</v>
+      <c r="C16" s="1">
+        <v>596.79999999999995</v>
       </c>
       <c r="D16" s="1">
+        <v>641</v>
+      </c>
+      <c r="E16" s="1">
+        <v>613</v>
+      </c>
+      <c r="F16" s="1">
+        <v>637</v>
+      </c>
+      <c r="G16" s="1">
+        <v>609</v>
+      </c>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1">
         <v>596.79999999999995</v>
       </c>
-      <c r="E16" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C16, [1]stats!$C$4:$N$4,0))</f>
-        <v>641</v>
-      </c>
-      <c r="F16" s="1">
-        <v>613</v>
-      </c>
-      <c r="G16" s="1">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J16" s="1"/>
+      <c r="K16" s="1">
+        <v>596.79999999999995</v>
+      </c>
+      <c r="L16" s="1">
+        <v>15000</v>
+      </c>
+      <c r="M16" s="1">
+        <v>18000</v>
+      </c>
+      <c r="N16" s="1">
+        <v>596.79999999999995</v>
+      </c>
+      <c r="O16" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>11</v>
       </c>
       <c r="B17" t="s">
         <v>13</v>
       </c>
-      <c r="C17" t="s">
-        <v>30</v>
+      <c r="C17" s="1">
+        <v>1335</v>
       </c>
       <c r="D17" s="1">
-        <v>1335</v>
+        <v>1569</v>
       </c>
       <c r="E17" s="1">
-        <f>INDEX([1]stats!$C$10:$N$10,MATCH($C17, [1]stats!$C$4:$N$4,0))</f>
-        <v>1569</v>
+        <v>1450</v>
       </c>
       <c r="F17" s="1">
-        <v>1450</v>
-      </c>
-      <c r="G17" s="1">
         <v>1563.5</v>
       </c>
+      <c r="G17">
+        <v>1425</v>
+      </c>
+      <c r="H17">
+        <v>1395</v>
+      </c>
+      <c r="J17" s="1">
+        <v>1558.5</v>
+      </c>
+      <c r="K17">
+        <v>1541</v>
+      </c>
+      <c r="L17" s="1">
+        <v>10000</v>
+      </c>
+      <c r="M17" s="1">
+        <v>17000</v>
+      </c>
+      <c r="N17" s="1">
+        <v>1541</v>
+      </c>
+      <c r="O17" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="K20" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:H17" xr:uid="{D5329979-E54C-48B7-8E55-3C9F10950753}"/>
+  <autoFilter ref="A6:P17" xr:uid="{D5329979-E54C-48B7-8E55-3C9F10950753}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="90" verticalDpi="90" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>